<commit_message>
fix: ensure all HOLIDAY column merges have center/center alignment on top-left cell
Re-merge all E column merge ranges and re-apply horizontal=center
vertical=center alignment to ensure HOLIDAY appears centered in merged block.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/lateness-book.xlsx
+++ b/src/lateness-book.xlsx
@@ -1099,7 +1099,7 @@
           <t>REASON</t>
         </is>
       </c>
-      <c r="E39" s="4" t="n"/>
+      <c r="E39" s="45" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -1313,7 +1313,7 @@
           <t>REASON</t>
         </is>
       </c>
-      <c r="E57" s="4" t="n"/>
+      <c r="E57" s="45" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -1523,7 +1523,7 @@
           <t>REASON</t>
         </is>
       </c>
-      <c r="E75" s="4" t="n"/>
+      <c r="E75" s="45" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">

</xml_diff>

<commit_message>
fix: re-merge all E column holiday ranges with explicit center/center alignment on top cell
Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/lateness-book.xlsx
+++ b/src/lateness-book.xlsx
@@ -19,7 +19,7 @@
     <numFmt numFmtId="164" formatCode="[$-409]h:mm\ AM/PM;@"/>
     <numFmt numFmtId="165" formatCode="[$GHC]\ #,##0.00"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -38,6 +38,10 @@
       <family val="1"/>
       <b val="1"/>
       <color theme="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
       <sz val="12"/>
     </font>
   </fonts>
@@ -218,7 +222,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -319,6 +323,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -681,7 +691,7 @@
           <t>REASON</t>
         </is>
       </c>
-      <c r="E3" s="26" t="inlineStr">
+      <c r="E3" s="46" t="inlineStr">
         <is>
           <t>HOLIDAY</t>
         </is>
@@ -891,7 +901,7 @@
           <t>REASON</t>
         </is>
       </c>
-      <c r="E21" s="45" t="n"/>
+      <c r="E21" s="47" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -1099,7 +1109,7 @@
           <t>REASON</t>
         </is>
       </c>
-      <c r="E39" s="45" t="n"/>
+      <c r="E39" s="47" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -1313,7 +1323,7 @@
           <t>REASON</t>
         </is>
       </c>
-      <c r="E57" s="45" t="n"/>
+      <c r="E57" s="47" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -1523,7 +1533,7 @@
           <t>REASON</t>
         </is>
       </c>
-      <c r="E75" s="45" t="n"/>
+      <c r="E75" s="47" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
@@ -1885,8 +1895,8 @@
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="E57:E72"/>
+    <mergeCell ref="A55:E56"/>
     <mergeCell ref="E75:E90"/>
-    <mergeCell ref="A55:E56"/>
     <mergeCell ref="A37:E38"/>
     <mergeCell ref="A73:E74"/>
     <mergeCell ref="E3:E18"/>

</xml_diff>

<commit_message>
fix: copy exact E3 formatting from original LATENESS BOOK — font Times New Roman bold 12, center/center alignment, full border and fill styling
Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/lateness-book.xlsx
+++ b/src/lateness-book.xlsx
@@ -691,7 +691,7 @@
           <t>REASON</t>
         </is>
       </c>
-      <c r="E3" s="46" t="inlineStr">
+      <c r="E3" s="26" t="inlineStr">
         <is>
           <t>HOLIDAY</t>
         </is>
@@ -901,7 +901,7 @@
           <t>REASON</t>
         </is>
       </c>
-      <c r="E21" s="47" t="n"/>
+      <c r="E21" s="26" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -1109,7 +1109,7 @@
           <t>REASON</t>
         </is>
       </c>
-      <c r="E39" s="47" t="n"/>
+      <c r="E39" s="26" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -1323,7 +1323,7 @@
           <t>REASON</t>
         </is>
       </c>
-      <c r="E57" s="47" t="n"/>
+      <c r="E57" s="26" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -1533,7 +1533,7 @@
           <t>REASON</t>
         </is>
       </c>
-      <c r="E75" s="47" t="n"/>
+      <c r="E75" s="26" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
@@ -1895,8 +1895,8 @@
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="E57:E72"/>
+    <mergeCell ref="E75:E90"/>
     <mergeCell ref="A55:E56"/>
-    <mergeCell ref="E75:E90"/>
     <mergeCell ref="A37:E38"/>
     <mergeCell ref="A73:E74"/>
     <mergeCell ref="E3:E18"/>

</xml_diff>

<commit_message>
fix: copy full E column cell styling from original — value, alignment center/center, Times New Roman 12pt bold, border, fill for all day header rows
Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/lateness-book.xlsx
+++ b/src/lateness-book.xlsx
@@ -901,7 +901,7 @@
           <t>REASON</t>
         </is>
       </c>
-      <c r="E21" s="26" t="n"/>
+      <c r="E21" s="45" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -1109,7 +1109,7 @@
           <t>REASON</t>
         </is>
       </c>
-      <c r="E39" s="26" t="n"/>
+      <c r="E39" s="45" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -1323,7 +1323,7 @@
           <t>REASON</t>
         </is>
       </c>
-      <c r="E57" s="26" t="n"/>
+      <c r="E57" s="45" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -1533,7 +1533,7 @@
           <t>REASON</t>
         </is>
       </c>
-      <c r="E75" s="26" t="n"/>
+      <c r="E75" s="45" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">

</xml_diff>